<commit_message>
Fix Chinese font display issue and update scheduled run time
</commit_message>
<xml_diff>
--- a/IC期货基差数据_最终版.xlsx
+++ b/IC期货基差数据_最终版.xlsx
@@ -446,7 +446,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-12-26</t>
+          <t>2025-12-29</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>41</v>
+        <v>42.6</v>
       </c>
       <c r="D2" t="n">
-        <v>34.2</v>
+        <v>42.5</v>
       </c>
       <c r="E2" t="n">
-        <v>50.44</v>
+        <v>52.8</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-12-29</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -476,19 +476,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>42.6</v>
+        <v>39.8</v>
       </c>
       <c r="D3" t="n">
-        <v>42.5</v>
+        <v>38.1</v>
       </c>
       <c r="E3" t="n">
-        <v>52.8</v>
+        <v>51.24</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -497,19 +497,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>39.8</v>
+        <v>47.8</v>
       </c>
       <c r="D4" t="n">
-        <v>38.1</v>
+        <v>46.4</v>
       </c>
       <c r="E4" t="n">
-        <v>51.24</v>
+        <v>56.04</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-12-31</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -518,19 +518,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>47.8</v>
+        <v>40</v>
       </c>
       <c r="D5" t="n">
-        <v>46.4</v>
+        <v>34.4</v>
       </c>
       <c r="E5" t="n">
-        <v>56.04</v>
+        <v>49.56</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -539,19 +539,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>40</v>
+        <v>30.4</v>
       </c>
       <c r="D6" t="n">
-        <v>34.4</v>
+        <v>24.8</v>
       </c>
       <c r="E6" t="n">
-        <v>49.56</v>
+        <v>44.52</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -560,19 +560,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>30.4</v>
+        <v>38.2</v>
       </c>
       <c r="D7" t="n">
-        <v>24.8</v>
+        <v>33.5</v>
       </c>
       <c r="E7" t="n">
-        <v>44.52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -581,19 +581,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>38.2</v>
+        <v>40.2</v>
       </c>
       <c r="D8" t="n">
-        <v>33.5</v>
+        <v>37.5</v>
       </c>
       <c r="E8" t="n">
-        <v>48</v>
+        <v>49.68</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -602,19 +602,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>40.2</v>
+        <v>30</v>
       </c>
       <c r="D9" t="n">
-        <v>37.5</v>
+        <v>25.2</v>
       </c>
       <c r="E9" t="n">
-        <v>49.68</v>
+        <v>44.52</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -623,19 +623,19 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>30</v>
+        <v>15.6</v>
       </c>
       <c r="D10" t="n">
-        <v>25.2</v>
+        <v>18.6</v>
       </c>
       <c r="E10" t="n">
-        <v>44.52</v>
+        <v>38.08</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -644,19 +644,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>15.6</v>
+        <v>22.2</v>
       </c>
       <c r="D11" t="n">
-        <v>18.6</v>
+        <v>20.8</v>
       </c>
       <c r="E11" t="n">
-        <v>38.08</v>
+        <v>37.52</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -665,19 +665,19 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>22.2</v>
+        <v>2.4</v>
       </c>
       <c r="D12" t="n">
-        <v>20.8</v>
+        <v>11.6</v>
       </c>
       <c r="E12" t="n">
-        <v>37.52</v>
+        <v>36.44</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-15</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -686,40 +686,40 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2.4</v>
+        <v>-2.6</v>
       </c>
       <c r="D13" t="n">
-        <v>11.6</v>
+        <v>5.3</v>
       </c>
       <c r="E13" t="n">
-        <v>36.44</v>
+        <v>29.8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IC2601</t>
+          <t>IC2602</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>-2.6</v>
+        <v>15.8</v>
       </c>
       <c r="D14" t="n">
-        <v>5.3</v>
+        <v>33.45</v>
       </c>
       <c r="E14" t="n">
-        <v>29.8</v>
+        <v>36.83</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -728,19 +728,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>15.8</v>
+        <v>9</v>
       </c>
       <c r="D15" t="n">
-        <v>33.45</v>
+        <v>28.95</v>
       </c>
       <c r="E15" t="n">
-        <v>36.83</v>
+        <v>33.37</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -749,19 +749,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>9</v>
+        <v>2.2</v>
       </c>
       <c r="D16" t="n">
-        <v>28.95</v>
+        <v>25.85</v>
       </c>
       <c r="E16" t="n">
-        <v>33.37</v>
+        <v>30.74</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -770,19 +770,19 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2.2</v>
+        <v>4</v>
       </c>
       <c r="D17" t="n">
-        <v>25.85</v>
+        <v>23.6</v>
       </c>
       <c r="E17" t="n">
-        <v>30.74</v>
+        <v>29.83</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-01-23</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -791,19 +791,19 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
+        <v>-2</v>
       </c>
       <c r="D18" t="n">
+        <v>19.35</v>
+      </c>
+      <c r="E18" t="n">
         <v>23.6</v>
-      </c>
-      <c r="E18" t="n">
-        <v>29.83</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-01-23</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -812,19 +812,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>-2</v>
+        <v>15.2</v>
       </c>
       <c r="D19" t="n">
-        <v>19.35</v>
+        <v>28.55</v>
       </c>
       <c r="E19" t="n">
-        <v>23.6</v>
+        <v>32.14</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-01-26</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,19 +833,19 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>15.2</v>
+        <v>6.6</v>
       </c>
       <c r="D20" t="n">
-        <v>28.55</v>
+        <v>19.8</v>
       </c>
       <c r="E20" t="n">
-        <v>32.14</v>
+        <v>26.26</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -854,19 +854,19 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>6.6</v>
+        <v>1.2</v>
       </c>
       <c r="D21" t="n">
-        <v>19.8</v>
+        <v>12.1</v>
       </c>
       <c r="E21" t="n">
-        <v>26.26</v>
+        <v>22.03</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -875,19 +875,19 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1.2</v>
+        <v>13.6</v>
       </c>
       <c r="D22" t="n">
-        <v>12.1</v>
+        <v>17.05</v>
       </c>
       <c r="E22" t="n">
-        <v>22.03</v>
+        <v>22.46</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -896,19 +896,19 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>13.6</v>
+        <v>14.8</v>
       </c>
       <c r="D23" t="n">
-        <v>17.05</v>
+        <v>19.3</v>
       </c>
       <c r="E23" t="n">
-        <v>22.46</v>
+        <v>23.89</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -917,19 +917,19 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>14.8</v>
+        <v>47.8</v>
       </c>
       <c r="D24" t="n">
-        <v>19.3</v>
+        <v>46.45</v>
       </c>
       <c r="E24" t="n">
-        <v>23.89</v>
+        <v>43.43</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -938,19 +938,19 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>47.8</v>
+        <v>13.8</v>
       </c>
       <c r="D25" t="n">
-        <v>46.45</v>
+        <v>26.55</v>
       </c>
       <c r="E25" t="n">
-        <v>43.43</v>
+        <v>28.69</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -959,19 +959,19 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>13.8</v>
+        <v>7.4</v>
       </c>
       <c r="D26" t="n">
-        <v>26.55</v>
+        <v>26.25</v>
       </c>
       <c r="E26" t="n">
-        <v>28.69</v>
+        <v>30.86</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -980,19 +980,19 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>7.4</v>
+        <v>24.8</v>
       </c>
       <c r="D27" t="n">
-        <v>26.25</v>
+        <v>33.2</v>
       </c>
       <c r="E27" t="n">
-        <v>30.86</v>
+        <v>34.97</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-02-05</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1001,19 +1001,19 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>24.8</v>
+        <v>23.2</v>
       </c>
       <c r="D28" t="n">
-        <v>33.2</v>
+        <v>31.25</v>
       </c>
       <c r="E28" t="n">
-        <v>34.97</v>
+        <v>34.37</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1022,19 +1022,19 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>23.2</v>
+        <v>10.4</v>
       </c>
       <c r="D29" t="n">
-        <v>31.25</v>
+        <v>26.7</v>
       </c>
       <c r="E29" t="n">
-        <v>34.37</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1043,19 +1043,19 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>10.4</v>
+        <v>18.2</v>
       </c>
       <c r="D30" t="n">
-        <v>26.7</v>
+        <v>29.95</v>
       </c>
       <c r="E30" t="n">
-        <v>32.4</v>
+        <v>35</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1064,19 +1064,19 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>18.2</v>
+        <v>6</v>
       </c>
       <c r="D31" t="n">
-        <v>29.95</v>
+        <v>26.8</v>
       </c>
       <c r="E31" t="n">
-        <v>35</v>
+        <v>32.14</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1085,19 +1085,19 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>6</v>
+        <v>-0.6</v>
       </c>
       <c r="D32" t="n">
-        <v>26.8</v>
+        <v>24.55</v>
       </c>
       <c r="E32" t="n">
-        <v>32.14</v>
+        <v>30.51</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1106,40 +1106,40 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>-0.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="D33" t="n">
-        <v>24.55</v>
+        <v>29.4</v>
       </c>
       <c r="E33" t="n">
-        <v>30.51</v>
+        <v>33.54</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>IC2602</t>
+          <t>IC2603</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>8.199999999999999</v>
+        <v>14.2</v>
       </c>
       <c r="D34" t="n">
-        <v>29.4</v>
+        <v>30.53</v>
       </c>
       <c r="E34" t="n">
-        <v>33.54</v>
+        <v>35.33</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1148,19 +1148,19 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>14.2</v>
+        <v>22.4</v>
       </c>
       <c r="D35" t="n">
-        <v>30.53</v>
+        <v>36.67</v>
       </c>
       <c r="E35" t="n">
-        <v>35.33</v>
+        <v>39.87</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1169,19 +1169,19 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>22.4</v>
+        <v>25.2</v>
       </c>
       <c r="D36" t="n">
-        <v>36.67</v>
+        <v>40.07</v>
       </c>
       <c r="E36" t="n">
-        <v>39.87</v>
+        <v>44.87</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1190,19 +1190,19 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>25.2</v>
+        <v>24</v>
       </c>
       <c r="D37" t="n">
-        <v>40.07</v>
+        <v>41.67</v>
       </c>
       <c r="E37" t="n">
-        <v>44.87</v>
+        <v>46</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1211,19 +1211,19 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>24</v>
+        <v>51.4</v>
       </c>
       <c r="D38" t="n">
-        <v>41.67</v>
+        <v>43.33</v>
       </c>
       <c r="E38" t="n">
-        <v>46</v>
+        <v>45.5</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1232,19 +1232,19 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>51.4</v>
+        <v>27.2</v>
       </c>
       <c r="D39" t="n">
-        <v>43.33</v>
+        <v>47.87</v>
       </c>
       <c r="E39" t="n">
-        <v>45.5</v>
+        <v>49.63</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-03-05</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1253,19 +1253,19 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>27.2</v>
+        <v>34.6</v>
       </c>
       <c r="D40" t="n">
-        <v>47.87</v>
+        <v>56</v>
       </c>
       <c r="E40" t="n">
-        <v>49.63</v>
+        <v>55.67</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1274,19 +1274,19 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>34.6</v>
+        <v>39.4</v>
       </c>
       <c r="D41" t="n">
-        <v>56</v>
+        <v>57.27</v>
       </c>
       <c r="E41" t="n">
-        <v>55.67</v>
+        <v>57.47</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1295,19 +1295,19 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>39.4</v>
+        <v>47</v>
       </c>
       <c r="D42" t="n">
-        <v>57.27</v>
+        <v>61.73</v>
       </c>
       <c r="E42" t="n">
-        <v>57.47</v>
+        <v>60.87</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1316,19 +1316,19 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>47</v>
+        <v>38.6</v>
       </c>
       <c r="D43" t="n">
-        <v>61.73</v>
+        <v>51.53</v>
       </c>
       <c r="E43" t="n">
-        <v>60.87</v>
+        <v>51.73</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-11</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1337,19 +1337,19 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>38.6</v>
+        <v>43.2</v>
       </c>
       <c r="D44" t="n">
-        <v>51.53</v>
+        <v>53.53</v>
       </c>
       <c r="E44" t="n">
-        <v>51.73</v>
+        <v>53.6</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1358,19 +1358,19 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>43.2</v>
+        <v>44.6</v>
       </c>
       <c r="D45" t="n">
-        <v>53.53</v>
+        <v>57.93</v>
       </c>
       <c r="E45" t="n">
-        <v>53.6</v>
+        <v>55.2</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1379,19 +1379,19 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>44.6</v>
+        <v>48.8</v>
       </c>
       <c r="D46" t="n">
-        <v>57.93</v>
+        <v>61</v>
       </c>
       <c r="E46" t="n">
-        <v>55.2</v>
+        <v>58.4</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1400,19 +1400,19 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>48.8</v>
+        <v>41.6</v>
       </c>
       <c r="D47" t="n">
-        <v>61</v>
+        <v>58.33</v>
       </c>
       <c r="E47" t="n">
-        <v>58.4</v>
+        <v>56.6</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-17</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1421,19 +1421,19 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>41.6</v>
+        <v>50</v>
       </c>
       <c r="D48" t="n">
-        <v>58.33</v>
+        <v>63.4</v>
       </c>
       <c r="E48" t="n">
-        <v>56.6</v>
+        <v>61.3</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-03-17</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1442,19 +1442,19 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="D49" t="n">
-        <v>63.4</v>
+        <v>67.2</v>
       </c>
       <c r="E49" t="n">
-        <v>61.3</v>
+        <v>61.97</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1463,40 +1463,40 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>55</v>
+        <v>64.2</v>
       </c>
       <c r="D50" t="n">
-        <v>67.2</v>
+        <v>71.8</v>
       </c>
       <c r="E50" t="n">
-        <v>61.97</v>
+        <v>65.37</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>IC2603</t>
+          <t>IC2604</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>64.2</v>
+        <v>50</v>
       </c>
       <c r="D51" t="n">
-        <v>71.8</v>
+        <v>76.3</v>
       </c>
       <c r="E51" t="n">
-        <v>65.37</v>
+        <v>67.72</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1505,19 +1505,19 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>50</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="D52" t="n">
-        <v>76.3</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="E52" t="n">
-        <v>67.72</v>
+        <v>63.08</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1526,13 +1526,13 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>70.59999999999999</v>
+        <v>55.6</v>
       </c>
       <c r="D53" t="n">
-        <v>72.59999999999999</v>
+        <v>77.8</v>
       </c>
       <c r="E53" t="n">
-        <v>63.08</v>
+        <v>66.12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>